<commit_message>
Add subtype consensus mutation summaries
</commit_message>
<xml_diff>
--- a/Reference_seqs/HCV_Subtype_Ref_vs_Comet_Subtype_Consensus_Aligned_NS3.xlsx
+++ b/Reference_seqs/HCV_Subtype_Ref_vs_Comet_Subtype_Consensus_Aligned_NS3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S384"/>
+  <dimension ref="A1:T384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -439,6 +439,7 @@
     <col width="5" customWidth="1" min="17" max="17"/>
     <col width="5" customWidth="1" min="18" max="18"/>
     <col width="5" customWidth="1" min="19" max="19"/>
+    <col width="50" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -508,6 +509,11 @@
       <c r="S2" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T2" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -627,21 +633,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
     </row>
     <row r="5"/>
     <row r="6">
@@ -710,6 +701,11 @@
       <c r="S6" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T6" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -829,21 +825,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9"/>
     <row r="10">
@@ -912,6 +893,11 @@
       <c r="S10" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T10" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1036,24 +1022,36 @@
           <t>V</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <r>
+            <t>L36V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>99</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>I170V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>68</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="13"/>
     <row r="14">
@@ -1122,6 +1120,11 @@
       <c r="S14" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T14" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1241,21 +1244,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
     </row>
     <row r="17"/>
     <row r="18">
@@ -1324,6 +1312,11 @@
       <c r="S18" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T18" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1443,21 +1436,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="inlineStr"/>
-      <c r="R20" t="inlineStr"/>
-      <c r="S20" t="inlineStr"/>
     </row>
     <row r="21"/>
     <row r="22">
@@ -1526,6 +1504,11 @@
       <c r="S22" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T22" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1645,21 +1628,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25"/>
     <row r="26">
@@ -1728,6 +1696,11 @@
       <c r="S26" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T26" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1847,29 +1820,41 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
           <t>Q</t>
         </is>
       </c>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <r>
+            <t>S54T</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>93</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>K80Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>73</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="29"/>
     <row r="30">
@@ -1938,6 +1923,11 @@
       <c r="S30" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T30" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2057,21 +2047,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
     </row>
     <row r="33"/>
     <row r="34">
@@ -2140,6 +2115,11 @@
       <c r="S34" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T34" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2259,25 +2239,24 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr">
+        <is>
+          <r>
+            <t>T122N</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>78</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="37"/>
     <row r="38">
@@ -2346,6 +2325,11 @@
       <c r="S38" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T38" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2465,21 +2449,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
     </row>
     <row r="41"/>
     <row r="42">
@@ -2548,6 +2517,11 @@
       <c r="S42" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T42" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2667,21 +2641,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
-      <c r="S44" t="inlineStr"/>
     </row>
     <row r="45"/>
     <row r="46">
@@ -2750,6 +2709,11 @@
       <c r="S46" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T46" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2869,21 +2833,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
-      <c r="S48" t="inlineStr"/>
     </row>
     <row r="49"/>
     <row r="50">
@@ -2952,6 +2901,11 @@
       <c r="S50" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T50" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3071,21 +3025,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
     </row>
     <row r="53"/>
     <row r="54">
@@ -3154,6 +3093,11 @@
       <c r="S54" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T54" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3273,21 +3217,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
     </row>
     <row r="57"/>
     <row r="58">
@@ -3356,6 +3285,11 @@
       <c r="S58" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T58" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3475,25 +3409,24 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="S60" t="inlineStr"/>
+      <c r="T60" t="inlineStr">
+        <is>
+          <r>
+            <t>I170V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>93</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="61"/>
     <row r="62">
@@ -3562,6 +3495,11 @@
       <c r="S62" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T62" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3681,21 +3619,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr"/>
-      <c r="R64" t="inlineStr"/>
-      <c r="S64" t="inlineStr"/>
     </row>
     <row r="65"/>
     <row r="66">
@@ -3764,6 +3687,11 @@
       <c r="S66" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T66" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3883,21 +3811,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
-      <c r="R68" t="inlineStr"/>
-      <c r="S68" t="inlineStr"/>
     </row>
     <row r="69"/>
     <row r="70">
@@ -3966,6 +3879,11 @@
       <c r="S70" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T70" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4085,21 +4003,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
     </row>
     <row r="73"/>
     <row r="74">
@@ -4168,6 +4071,11 @@
       <c r="S74" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T74" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4287,21 +4195,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
-      <c r="O76" t="inlineStr"/>
-      <c r="P76" t="inlineStr"/>
-      <c r="Q76" t="inlineStr"/>
-      <c r="R76" t="inlineStr"/>
-      <c r="S76" t="inlineStr"/>
     </row>
     <row r="77"/>
     <row r="78">
@@ -4370,6 +4263,11 @@
       <c r="S78" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T78" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4489,21 +4387,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="inlineStr"/>
-      <c r="O80" t="inlineStr"/>
-      <c r="P80" t="inlineStr"/>
-      <c r="Q80" t="inlineStr"/>
-      <c r="R80" t="inlineStr"/>
-      <c r="S80" t="inlineStr"/>
     </row>
     <row r="81"/>
     <row r="82">
@@ -4572,6 +4455,11 @@
       <c r="S82" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T82" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4691,21 +4579,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
-      <c r="P84" t="inlineStr"/>
-      <c r="Q84" t="inlineStr"/>
-      <c r="R84" t="inlineStr"/>
-      <c r="S84" t="inlineStr"/>
     </row>
     <row r="85"/>
     <row r="86">
@@ -4774,6 +4647,11 @@
       <c r="S86" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T86" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4893,21 +4771,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
-      <c r="P88" t="inlineStr"/>
-      <c r="Q88" t="inlineStr"/>
-      <c r="R88" t="inlineStr"/>
-      <c r="S88" t="inlineStr"/>
     </row>
     <row r="89"/>
     <row r="90">
@@ -4976,6 +4839,11 @@
       <c r="S90" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T90" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5095,21 +4963,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="inlineStr"/>
-      <c r="O92" t="inlineStr"/>
-      <c r="P92" t="inlineStr"/>
-      <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
-      <c r="S92" t="inlineStr"/>
     </row>
     <row r="93"/>
     <row r="94">
@@ -5178,6 +5031,11 @@
       <c r="S94" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T94" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5297,21 +5155,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
-      <c r="N96" t="inlineStr"/>
-      <c r="O96" t="inlineStr"/>
-      <c r="P96" t="inlineStr"/>
-      <c r="Q96" t="inlineStr"/>
-      <c r="R96" t="inlineStr"/>
-      <c r="S96" t="inlineStr"/>
     </row>
     <row r="97"/>
     <row r="98">
@@ -5380,6 +5223,11 @@
       <c r="S98" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T98" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5499,21 +5347,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
-      <c r="N100" t="inlineStr"/>
-      <c r="O100" t="inlineStr"/>
-      <c r="P100" t="inlineStr"/>
-      <c r="Q100" t="inlineStr"/>
-      <c r="R100" t="inlineStr"/>
-      <c r="S100" t="inlineStr"/>
     </row>
     <row r="101"/>
     <row r="102">
@@ -5582,6 +5415,11 @@
       <c r="S102" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T102" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5701,21 +5539,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
-      <c r="N104" t="inlineStr"/>
-      <c r="O104" t="inlineStr"/>
-      <c r="P104" t="inlineStr"/>
-      <c r="Q104" t="inlineStr"/>
-      <c r="R104" t="inlineStr"/>
-      <c r="S104" t="inlineStr"/>
     </row>
     <row r="105"/>
     <row r="106">
@@ -5784,6 +5607,11 @@
       <c r="S106" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T106" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5903,21 +5731,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
-      <c r="M108" t="inlineStr"/>
-      <c r="N108" t="inlineStr"/>
-      <c r="O108" t="inlineStr"/>
-      <c r="P108" t="inlineStr"/>
-      <c r="Q108" t="inlineStr"/>
-      <c r="R108" t="inlineStr"/>
-      <c r="S108" t="inlineStr"/>
     </row>
     <row r="109"/>
     <row r="110">
@@ -5986,6 +5799,11 @@
       <c r="S110" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T110" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6105,21 +5923,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
-      <c r="M112" t="inlineStr"/>
-      <c r="N112" t="inlineStr"/>
-      <c r="O112" t="inlineStr"/>
-      <c r="P112" t="inlineStr"/>
-      <c r="Q112" t="inlineStr"/>
-      <c r="R112" t="inlineStr"/>
-      <c r="S112" t="inlineStr"/>
     </row>
     <row r="113"/>
     <row r="114">
@@ -6188,6 +5991,11 @@
       <c r="S114" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T114" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6307,21 +6115,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
-      <c r="M116" t="inlineStr"/>
-      <c r="N116" t="inlineStr"/>
-      <c r="O116" t="inlineStr"/>
-      <c r="P116" t="inlineStr"/>
-      <c r="Q116" t="inlineStr"/>
-      <c r="R116" t="inlineStr"/>
-      <c r="S116" t="inlineStr"/>
     </row>
     <row r="117"/>
     <row r="118">
@@ -6390,6 +6183,11 @@
       <c r="S118" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T118" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6509,21 +6307,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
-      <c r="M120" t="inlineStr"/>
-      <c r="N120" t="inlineStr"/>
-      <c r="O120" t="inlineStr"/>
-      <c r="P120" t="inlineStr"/>
-      <c r="Q120" t="inlineStr"/>
-      <c r="R120" t="inlineStr"/>
-      <c r="S120" t="inlineStr"/>
     </row>
     <row r="121"/>
     <row r="122">
@@ -6592,6 +6375,11 @@
       <c r="S122" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T122" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6711,21 +6499,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
-      <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
-      <c r="N124" t="inlineStr"/>
-      <c r="O124" t="inlineStr"/>
-      <c r="P124" t="inlineStr"/>
-      <c r="Q124" t="inlineStr"/>
-      <c r="R124" t="inlineStr"/>
-      <c r="S124" t="inlineStr"/>
     </row>
     <row r="125"/>
     <row r="126">
@@ -6794,6 +6567,11 @@
       <c r="S126" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T126" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6913,21 +6691,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr"/>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
-      <c r="M128" t="inlineStr"/>
-      <c r="N128" t="inlineStr"/>
-      <c r="O128" t="inlineStr"/>
-      <c r="P128" t="inlineStr"/>
-      <c r="Q128" t="inlineStr"/>
-      <c r="R128" t="inlineStr"/>
-      <c r="S128" t="inlineStr"/>
     </row>
     <row r="129"/>
     <row r="130">
@@ -6996,6 +6759,11 @@
       <c r="S130" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T130" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -7115,21 +6883,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
-      <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr"/>
-      <c r="H132" t="inlineStr"/>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
-      <c r="M132" t="inlineStr"/>
-      <c r="N132" t="inlineStr"/>
-      <c r="O132" t="inlineStr"/>
-      <c r="P132" t="inlineStr"/>
-      <c r="Q132" t="inlineStr"/>
-      <c r="R132" t="inlineStr"/>
-      <c r="S132" t="inlineStr"/>
     </row>
     <row r="133"/>
     <row r="134">
@@ -7198,6 +6951,11 @@
       <c r="S134" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T134" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -7317,21 +7075,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
-      <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr"/>
-      <c r="H136" t="inlineStr"/>
-      <c r="I136" t="inlineStr"/>
-      <c r="J136" t="inlineStr"/>
-      <c r="K136" t="inlineStr"/>
-      <c r="L136" t="inlineStr"/>
-      <c r="M136" t="inlineStr"/>
-      <c r="N136" t="inlineStr"/>
-      <c r="O136" t="inlineStr"/>
-      <c r="P136" t="inlineStr"/>
-      <c r="Q136" t="inlineStr"/>
-      <c r="R136" t="inlineStr"/>
-      <c r="S136" t="inlineStr"/>
     </row>
     <row r="137"/>
     <row r="138">
@@ -7400,6 +7143,11 @@
       <c r="S138" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T138" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -7519,23 +7267,22 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
-      <c r="F140" t="inlineStr"/>
-      <c r="G140" t="inlineStr"/>
-      <c r="H140" t="inlineStr"/>
-      <c r="I140" t="inlineStr"/>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
-      <c r="L140" t="inlineStr"/>
-      <c r="M140" t="inlineStr"/>
-      <c r="N140" t="inlineStr"/>
-      <c r="O140" t="inlineStr"/>
-      <c r="P140" t="inlineStr"/>
-      <c r="Q140" t="inlineStr"/>
-      <c r="R140" t="inlineStr"/>
       <c r="S140" t="inlineStr">
         <is>
           <t>S</t>
+        </is>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <r>
+            <t>N175S</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>NA</t>
+          </r>
         </is>
       </c>
     </row>
@@ -7606,6 +7353,11 @@
       <c r="S142" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T142" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7725,25 +7477,24 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
-      <c r="F144" t="inlineStr"/>
-      <c r="G144" t="inlineStr"/>
-      <c r="H144" t="inlineStr"/>
-      <c r="I144" t="inlineStr"/>
-      <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
-      <c r="L144" t="inlineStr"/>
-      <c r="M144" t="inlineStr"/>
-      <c r="N144" t="inlineStr"/>
       <c r="O144" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="P144" t="inlineStr"/>
-      <c r="Q144" t="inlineStr"/>
-      <c r="R144" t="inlineStr"/>
-      <c r="S144" t="inlineStr"/>
+      <c r="T144" t="inlineStr">
+        <is>
+          <r>
+            <t>I158V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>91</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="145"/>
     <row r="146">
@@ -7812,6 +7563,11 @@
       <c r="S146" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T146" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7931,21 +7687,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr"/>
-      <c r="H148" t="inlineStr"/>
-      <c r="I148" t="inlineStr"/>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
-      <c r="L148" t="inlineStr"/>
-      <c r="M148" t="inlineStr"/>
-      <c r="N148" t="inlineStr"/>
-      <c r="O148" t="inlineStr"/>
-      <c r="P148" t="inlineStr"/>
-      <c r="Q148" t="inlineStr"/>
-      <c r="R148" t="inlineStr"/>
-      <c r="S148" t="inlineStr"/>
     </row>
     <row r="149"/>
     <row r="150">
@@ -8014,6 +7755,11 @@
       <c r="S150" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T150" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -8133,21 +7879,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr"/>
-      <c r="H152" t="inlineStr"/>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
-      <c r="L152" t="inlineStr"/>
-      <c r="M152" t="inlineStr"/>
-      <c r="N152" t="inlineStr"/>
-      <c r="O152" t="inlineStr"/>
-      <c r="P152" t="inlineStr"/>
-      <c r="Q152" t="inlineStr"/>
-      <c r="R152" t="inlineStr"/>
-      <c r="S152" t="inlineStr"/>
     </row>
     <row r="153"/>
     <row r="154">
@@ -8216,6 +7947,11 @@
       <c r="S154" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T154" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -8335,21 +8071,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr"/>
-      <c r="H156" t="inlineStr"/>
-      <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
-      <c r="L156" t="inlineStr"/>
-      <c r="M156" t="inlineStr"/>
-      <c r="N156" t="inlineStr"/>
-      <c r="O156" t="inlineStr"/>
-      <c r="P156" t="inlineStr"/>
-      <c r="Q156" t="inlineStr"/>
-      <c r="R156" t="inlineStr"/>
-      <c r="S156" t="inlineStr"/>
     </row>
     <row r="157"/>
     <row r="158">
@@ -8418,6 +8139,11 @@
       <c r="S158" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T158" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -8537,21 +8263,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
-      <c r="F160" t="inlineStr"/>
-      <c r="G160" t="inlineStr"/>
-      <c r="H160" t="inlineStr"/>
-      <c r="I160" t="inlineStr"/>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
-      <c r="L160" t="inlineStr"/>
-      <c r="M160" t="inlineStr"/>
-      <c r="N160" t="inlineStr"/>
-      <c r="O160" t="inlineStr"/>
-      <c r="P160" t="inlineStr"/>
-      <c r="Q160" t="inlineStr"/>
-      <c r="R160" t="inlineStr"/>
-      <c r="S160" t="inlineStr"/>
     </row>
     <row r="161"/>
     <row r="162">
@@ -8620,6 +8331,11 @@
       <c r="S162" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T162" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -8739,21 +8455,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr"/>
-      <c r="H164" t="inlineStr"/>
-      <c r="I164" t="inlineStr"/>
-      <c r="J164" t="inlineStr"/>
-      <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
-      <c r="M164" t="inlineStr"/>
-      <c r="N164" t="inlineStr"/>
-      <c r="O164" t="inlineStr"/>
-      <c r="P164" t="inlineStr"/>
-      <c r="Q164" t="inlineStr"/>
-      <c r="R164" t="inlineStr"/>
-      <c r="S164" t="inlineStr"/>
     </row>
     <row r="165"/>
     <row r="166">
@@ -8822,6 +8523,11 @@
       <c r="S166" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T166" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8941,25 +8647,24 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr"/>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
-      <c r="H168" t="inlineStr"/>
-      <c r="I168" t="inlineStr"/>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
       <c r="L168" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-      <c r="M168" t="inlineStr"/>
-      <c r="N168" t="inlineStr"/>
-      <c r="O168" t="inlineStr"/>
-      <c r="P168" t="inlineStr"/>
-      <c r="Q168" t="inlineStr"/>
-      <c r="R168" t="inlineStr"/>
-      <c r="S168" t="inlineStr"/>
+      <c r="T168" t="inlineStr">
+        <is>
+          <r>
+            <t>S122G</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>50</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="169"/>
     <row r="170">
@@ -9028,6 +8733,11 @@
       <c r="S170" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T170" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -9147,21 +8857,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr"/>
-      <c r="F172" t="inlineStr"/>
-      <c r="G172" t="inlineStr"/>
-      <c r="H172" t="inlineStr"/>
-      <c r="I172" t="inlineStr"/>
-      <c r="J172" t="inlineStr"/>
-      <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
-      <c r="M172" t="inlineStr"/>
-      <c r="N172" t="inlineStr"/>
-      <c r="O172" t="inlineStr"/>
-      <c r="P172" t="inlineStr"/>
-      <c r="Q172" t="inlineStr"/>
-      <c r="R172" t="inlineStr"/>
-      <c r="S172" t="inlineStr"/>
     </row>
     <row r="173"/>
     <row r="174">
@@ -9230,6 +8925,11 @@
       <c r="S174" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T174" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -9349,21 +9049,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr"/>
-      <c r="F176" t="inlineStr"/>
-      <c r="G176" t="inlineStr"/>
-      <c r="H176" t="inlineStr"/>
-      <c r="I176" t="inlineStr"/>
-      <c r="J176" t="inlineStr"/>
-      <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
-      <c r="M176" t="inlineStr"/>
-      <c r="N176" t="inlineStr"/>
-      <c r="O176" t="inlineStr"/>
-      <c r="P176" t="inlineStr"/>
-      <c r="Q176" t="inlineStr"/>
-      <c r="R176" t="inlineStr"/>
-      <c r="S176" t="inlineStr"/>
     </row>
     <row r="177"/>
     <row r="178">
@@ -9432,6 +9117,11 @@
       <c r="S178" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T178" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -9551,21 +9241,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr"/>
-      <c r="H180" t="inlineStr"/>
-      <c r="I180" t="inlineStr"/>
-      <c r="J180" t="inlineStr"/>
-      <c r="K180" t="inlineStr"/>
-      <c r="L180" t="inlineStr"/>
-      <c r="M180" t="inlineStr"/>
-      <c r="N180" t="inlineStr"/>
-      <c r="O180" t="inlineStr"/>
-      <c r="P180" t="inlineStr"/>
-      <c r="Q180" t="inlineStr"/>
-      <c r="R180" t="inlineStr"/>
-      <c r="S180" t="inlineStr"/>
     </row>
     <row r="181"/>
     <row r="182">
@@ -9634,6 +9309,11 @@
       <c r="S182" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T182" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -9753,21 +9433,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr"/>
-      <c r="G184" t="inlineStr"/>
-      <c r="H184" t="inlineStr"/>
-      <c r="I184" t="inlineStr"/>
-      <c r="J184" t="inlineStr"/>
-      <c r="K184" t="inlineStr"/>
-      <c r="L184" t="inlineStr"/>
-      <c r="M184" t="inlineStr"/>
-      <c r="N184" t="inlineStr"/>
-      <c r="O184" t="inlineStr"/>
-      <c r="P184" t="inlineStr"/>
-      <c r="Q184" t="inlineStr"/>
-      <c r="R184" t="inlineStr"/>
-      <c r="S184" t="inlineStr"/>
     </row>
     <row r="185"/>
     <row r="186">
@@ -9836,6 +9501,11 @@
       <c r="S186" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T186" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -9955,21 +9625,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr"/>
-      <c r="F188" t="inlineStr"/>
-      <c r="G188" t="inlineStr"/>
-      <c r="H188" t="inlineStr"/>
-      <c r="I188" t="inlineStr"/>
-      <c r="J188" t="inlineStr"/>
-      <c r="K188" t="inlineStr"/>
-      <c r="L188" t="inlineStr"/>
-      <c r="M188" t="inlineStr"/>
-      <c r="N188" t="inlineStr"/>
-      <c r="O188" t="inlineStr"/>
-      <c r="P188" t="inlineStr"/>
-      <c r="Q188" t="inlineStr"/>
-      <c r="R188" t="inlineStr"/>
-      <c r="S188" t="inlineStr"/>
     </row>
     <row r="189"/>
     <row r="190">
@@ -10038,6 +9693,11 @@
       <c r="S190" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T190" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -10157,21 +9817,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr"/>
-      <c r="F192" t="inlineStr"/>
-      <c r="G192" t="inlineStr"/>
-      <c r="H192" t="inlineStr"/>
-      <c r="I192" t="inlineStr"/>
-      <c r="J192" t="inlineStr"/>
-      <c r="K192" t="inlineStr"/>
-      <c r="L192" t="inlineStr"/>
-      <c r="M192" t="inlineStr"/>
-      <c r="N192" t="inlineStr"/>
-      <c r="O192" t="inlineStr"/>
-      <c r="P192" t="inlineStr"/>
-      <c r="Q192" t="inlineStr"/>
-      <c r="R192" t="inlineStr"/>
-      <c r="S192" t="inlineStr"/>
     </row>
     <row r="193"/>
     <row r="194">
@@ -10240,6 +9885,11 @@
       <c r="S194" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T194" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -10359,21 +10009,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr"/>
-      <c r="F196" t="inlineStr"/>
-      <c r="G196" t="inlineStr"/>
-      <c r="H196" t="inlineStr"/>
-      <c r="I196" t="inlineStr"/>
-      <c r="J196" t="inlineStr"/>
-      <c r="K196" t="inlineStr"/>
-      <c r="L196" t="inlineStr"/>
-      <c r="M196" t="inlineStr"/>
-      <c r="N196" t="inlineStr"/>
-      <c r="O196" t="inlineStr"/>
-      <c r="P196" t="inlineStr"/>
-      <c r="Q196" t="inlineStr"/>
-      <c r="R196" t="inlineStr"/>
-      <c r="S196" t="inlineStr"/>
     </row>
     <row r="197"/>
     <row r="198">
@@ -10442,6 +10077,11 @@
       <c r="S198" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T198" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -10561,21 +10201,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr"/>
-      <c r="G200" t="inlineStr"/>
-      <c r="H200" t="inlineStr"/>
-      <c r="I200" t="inlineStr"/>
-      <c r="J200" t="inlineStr"/>
-      <c r="K200" t="inlineStr"/>
-      <c r="L200" t="inlineStr"/>
-      <c r="M200" t="inlineStr"/>
-      <c r="N200" t="inlineStr"/>
-      <c r="O200" t="inlineStr"/>
-      <c r="P200" t="inlineStr"/>
-      <c r="Q200" t="inlineStr"/>
-      <c r="R200" t="inlineStr"/>
-      <c r="S200" t="inlineStr"/>
     </row>
     <row r="201"/>
     <row r="202">
@@ -10644,6 +10269,11 @@
       <c r="S202" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T202" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -10763,21 +10393,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr"/>
-      <c r="F204" t="inlineStr"/>
-      <c r="G204" t="inlineStr"/>
-      <c r="H204" t="inlineStr"/>
-      <c r="I204" t="inlineStr"/>
-      <c r="J204" t="inlineStr"/>
-      <c r="K204" t="inlineStr"/>
-      <c r="L204" t="inlineStr"/>
-      <c r="M204" t="inlineStr"/>
-      <c r="N204" t="inlineStr"/>
-      <c r="O204" t="inlineStr"/>
-      <c r="P204" t="inlineStr"/>
-      <c r="Q204" t="inlineStr"/>
-      <c r="R204" t="inlineStr"/>
-      <c r="S204" t="inlineStr"/>
     </row>
     <row r="205"/>
     <row r="206">
@@ -10846,6 +10461,11 @@
       <c r="S206" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T206" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -10965,25 +10585,24 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
-      <c r="G208" t="inlineStr"/>
-      <c r="H208" t="inlineStr"/>
-      <c r="I208" t="inlineStr"/>
-      <c r="J208" t="inlineStr"/>
-      <c r="K208" t="inlineStr"/>
-      <c r="L208" t="inlineStr"/>
-      <c r="M208" t="inlineStr"/>
-      <c r="N208" t="inlineStr"/>
-      <c r="O208" t="inlineStr"/>
-      <c r="P208" t="inlineStr"/>
-      <c r="Q208" t="inlineStr"/>
       <c r="R208" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="S208" t="inlineStr"/>
+      <c r="T208" t="inlineStr">
+        <is>
+          <r>
+            <t>I170V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>80</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="209"/>
     <row r="210">
@@ -11052,6 +10671,11 @@
       <c r="S210" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T210" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -11171,21 +10795,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
-      <c r="G212" t="inlineStr"/>
-      <c r="H212" t="inlineStr"/>
-      <c r="I212" t="inlineStr"/>
-      <c r="J212" t="inlineStr"/>
-      <c r="K212" t="inlineStr"/>
-      <c r="L212" t="inlineStr"/>
-      <c r="M212" t="inlineStr"/>
-      <c r="N212" t="inlineStr"/>
-      <c r="O212" t="inlineStr"/>
-      <c r="P212" t="inlineStr"/>
-      <c r="Q212" t="inlineStr"/>
-      <c r="R212" t="inlineStr"/>
-      <c r="S212" t="inlineStr"/>
     </row>
     <row r="213"/>
     <row r="214">
@@ -11254,6 +10863,11 @@
       <c r="S214" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T214" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -11373,21 +10987,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr"/>
-      <c r="G216" t="inlineStr"/>
-      <c r="H216" t="inlineStr"/>
-      <c r="I216" t="inlineStr"/>
-      <c r="J216" t="inlineStr"/>
-      <c r="K216" t="inlineStr"/>
-      <c r="L216" t="inlineStr"/>
-      <c r="M216" t="inlineStr"/>
-      <c r="N216" t="inlineStr"/>
-      <c r="O216" t="inlineStr"/>
-      <c r="P216" t="inlineStr"/>
-      <c r="Q216" t="inlineStr"/>
-      <c r="R216" t="inlineStr"/>
-      <c r="S216" t="inlineStr"/>
     </row>
     <row r="217"/>
     <row r="218">
@@ -11456,6 +11055,11 @@
       <c r="S218" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T218" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -11575,21 +11179,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
-      <c r="G220" t="inlineStr"/>
-      <c r="H220" t="inlineStr"/>
-      <c r="I220" t="inlineStr"/>
-      <c r="J220" t="inlineStr"/>
-      <c r="K220" t="inlineStr"/>
-      <c r="L220" t="inlineStr"/>
-      <c r="M220" t="inlineStr"/>
-      <c r="N220" t="inlineStr"/>
-      <c r="O220" t="inlineStr"/>
-      <c r="P220" t="inlineStr"/>
-      <c r="Q220" t="inlineStr"/>
-      <c r="R220" t="inlineStr"/>
-      <c r="S220" t="inlineStr"/>
     </row>
     <row r="221"/>
     <row r="222">
@@ -11658,6 +11247,11 @@
       <c r="S222" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T222" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -11777,21 +11371,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
-      <c r="F224" t="inlineStr"/>
-      <c r="G224" t="inlineStr"/>
-      <c r="H224" t="inlineStr"/>
-      <c r="I224" t="inlineStr"/>
-      <c r="J224" t="inlineStr"/>
-      <c r="K224" t="inlineStr"/>
-      <c r="L224" t="inlineStr"/>
-      <c r="M224" t="inlineStr"/>
-      <c r="N224" t="inlineStr"/>
-      <c r="O224" t="inlineStr"/>
-      <c r="P224" t="inlineStr"/>
-      <c r="Q224" t="inlineStr"/>
-      <c r="R224" t="inlineStr"/>
-      <c r="S224" t="inlineStr"/>
     </row>
     <row r="225"/>
     <row r="226">
@@ -11860,6 +11439,11 @@
       <c r="S226" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T226" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -11979,21 +11563,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr"/>
-      <c r="G228" t="inlineStr"/>
-      <c r="H228" t="inlineStr"/>
-      <c r="I228" t="inlineStr"/>
-      <c r="J228" t="inlineStr"/>
-      <c r="K228" t="inlineStr"/>
-      <c r="L228" t="inlineStr"/>
-      <c r="M228" t="inlineStr"/>
-      <c r="N228" t="inlineStr"/>
-      <c r="O228" t="inlineStr"/>
-      <c r="P228" t="inlineStr"/>
-      <c r="Q228" t="inlineStr"/>
-      <c r="R228" t="inlineStr"/>
-      <c r="S228" t="inlineStr"/>
     </row>
     <row r="229"/>
     <row r="230">
@@ -12062,6 +11631,11 @@
       <c r="S230" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T230" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -12181,21 +11755,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr"/>
-      <c r="F232" t="inlineStr"/>
-      <c r="G232" t="inlineStr"/>
-      <c r="H232" t="inlineStr"/>
-      <c r="I232" t="inlineStr"/>
-      <c r="J232" t="inlineStr"/>
-      <c r="K232" t="inlineStr"/>
-      <c r="L232" t="inlineStr"/>
-      <c r="M232" t="inlineStr"/>
-      <c r="N232" t="inlineStr"/>
-      <c r="O232" t="inlineStr"/>
-      <c r="P232" t="inlineStr"/>
-      <c r="Q232" t="inlineStr"/>
-      <c r="R232" t="inlineStr"/>
-      <c r="S232" t="inlineStr"/>
     </row>
     <row r="233"/>
     <row r="234">
@@ -12264,6 +11823,11 @@
       <c r="S234" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T234" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -12383,21 +11947,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
-      <c r="F236" t="inlineStr"/>
-      <c r="G236" t="inlineStr"/>
-      <c r="H236" t="inlineStr"/>
-      <c r="I236" t="inlineStr"/>
-      <c r="J236" t="inlineStr"/>
-      <c r="K236" t="inlineStr"/>
-      <c r="L236" t="inlineStr"/>
-      <c r="M236" t="inlineStr"/>
-      <c r="N236" t="inlineStr"/>
-      <c r="O236" t="inlineStr"/>
-      <c r="P236" t="inlineStr"/>
-      <c r="Q236" t="inlineStr"/>
-      <c r="R236" t="inlineStr"/>
-      <c r="S236" t="inlineStr"/>
     </row>
     <row r="237"/>
     <row r="238">
@@ -12466,6 +12015,11 @@
       <c r="S238" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T238" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -12585,21 +12139,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr"/>
-      <c r="F240" t="inlineStr"/>
-      <c r="G240" t="inlineStr"/>
-      <c r="H240" t="inlineStr"/>
-      <c r="I240" t="inlineStr"/>
-      <c r="J240" t="inlineStr"/>
-      <c r="K240" t="inlineStr"/>
-      <c r="L240" t="inlineStr"/>
-      <c r="M240" t="inlineStr"/>
-      <c r="N240" t="inlineStr"/>
-      <c r="O240" t="inlineStr"/>
-      <c r="P240" t="inlineStr"/>
-      <c r="Q240" t="inlineStr"/>
-      <c r="R240" t="inlineStr"/>
-      <c r="S240" t="inlineStr"/>
     </row>
     <row r="241"/>
     <row r="242">
@@ -12668,6 +12207,11 @@
       <c r="S242" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T242" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -12787,21 +12331,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr"/>
-      <c r="F244" t="inlineStr"/>
-      <c r="G244" t="inlineStr"/>
-      <c r="H244" t="inlineStr"/>
-      <c r="I244" t="inlineStr"/>
-      <c r="J244" t="inlineStr"/>
-      <c r="K244" t="inlineStr"/>
-      <c r="L244" t="inlineStr"/>
-      <c r="M244" t="inlineStr"/>
-      <c r="N244" t="inlineStr"/>
-      <c r="O244" t="inlineStr"/>
-      <c r="P244" t="inlineStr"/>
-      <c r="Q244" t="inlineStr"/>
-      <c r="R244" t="inlineStr"/>
-      <c r="S244" t="inlineStr"/>
     </row>
     <row r="245"/>
     <row r="246">
@@ -12870,6 +12399,11 @@
       <c r="S246" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T246" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -12989,21 +12523,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr"/>
-      <c r="F248" t="inlineStr"/>
-      <c r="G248" t="inlineStr"/>
-      <c r="H248" t="inlineStr"/>
-      <c r="I248" t="inlineStr"/>
-      <c r="J248" t="inlineStr"/>
-      <c r="K248" t="inlineStr"/>
-      <c r="L248" t="inlineStr"/>
-      <c r="M248" t="inlineStr"/>
-      <c r="N248" t="inlineStr"/>
-      <c r="O248" t="inlineStr"/>
-      <c r="P248" t="inlineStr"/>
-      <c r="Q248" t="inlineStr"/>
-      <c r="R248" t="inlineStr"/>
-      <c r="S248" t="inlineStr"/>
     </row>
     <row r="249"/>
     <row r="250">
@@ -13072,6 +12591,11 @@
       <c r="S250" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T250" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -13191,21 +12715,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr"/>
-      <c r="F252" t="inlineStr"/>
-      <c r="G252" t="inlineStr"/>
-      <c r="H252" t="inlineStr"/>
-      <c r="I252" t="inlineStr"/>
-      <c r="J252" t="inlineStr"/>
-      <c r="K252" t="inlineStr"/>
-      <c r="L252" t="inlineStr"/>
-      <c r="M252" t="inlineStr"/>
-      <c r="N252" t="inlineStr"/>
-      <c r="O252" t="inlineStr"/>
-      <c r="P252" t="inlineStr"/>
-      <c r="Q252" t="inlineStr"/>
-      <c r="R252" t="inlineStr"/>
-      <c r="S252" t="inlineStr"/>
     </row>
     <row r="253"/>
     <row r="254">
@@ -13274,6 +12783,11 @@
       <c r="S254" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T254" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -13393,21 +12907,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr"/>
-      <c r="F256" t="inlineStr"/>
-      <c r="G256" t="inlineStr"/>
-      <c r="H256" t="inlineStr"/>
-      <c r="I256" t="inlineStr"/>
-      <c r="J256" t="inlineStr"/>
-      <c r="K256" t="inlineStr"/>
-      <c r="L256" t="inlineStr"/>
-      <c r="M256" t="inlineStr"/>
-      <c r="N256" t="inlineStr"/>
-      <c r="O256" t="inlineStr"/>
-      <c r="P256" t="inlineStr"/>
-      <c r="Q256" t="inlineStr"/>
-      <c r="R256" t="inlineStr"/>
-      <c r="S256" t="inlineStr"/>
     </row>
     <row r="257"/>
     <row r="258">
@@ -13476,6 +12975,11 @@
       <c r="S258" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T258" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -13595,12 +13099,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E260" t="inlineStr"/>
-      <c r="F260" t="inlineStr"/>
-      <c r="G260" t="inlineStr"/>
-      <c r="H260" t="inlineStr"/>
-      <c r="I260" t="inlineStr"/>
-      <c r="J260" t="inlineStr"/>
       <c r="K260" t="inlineStr">
         <is>
           <t>K</t>
@@ -13611,13 +13109,31 @@
           <t>N</t>
         </is>
       </c>
-      <c r="M260" t="inlineStr"/>
-      <c r="N260" t="inlineStr"/>
-      <c r="O260" t="inlineStr"/>
-      <c r="P260" t="inlineStr"/>
-      <c r="Q260" t="inlineStr"/>
-      <c r="R260" t="inlineStr"/>
-      <c r="S260" t="inlineStr"/>
+      <c r="T260" t="inlineStr">
+        <is>
+          <r>
+            <t>L80K</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>97</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>S122N</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>77</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="261"/>
     <row r="262">
@@ -13686,6 +13202,11 @@
       <c r="S262" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T262" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -13805,21 +13326,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E264" t="inlineStr"/>
-      <c r="F264" t="inlineStr"/>
-      <c r="G264" t="inlineStr"/>
-      <c r="H264" t="inlineStr"/>
-      <c r="I264" t="inlineStr"/>
-      <c r="J264" t="inlineStr"/>
-      <c r="K264" t="inlineStr"/>
-      <c r="L264" t="inlineStr"/>
-      <c r="M264" t="inlineStr"/>
-      <c r="N264" t="inlineStr"/>
-      <c r="O264" t="inlineStr"/>
-      <c r="P264" t="inlineStr"/>
-      <c r="Q264" t="inlineStr"/>
-      <c r="R264" t="inlineStr"/>
-      <c r="S264" t="inlineStr"/>
     </row>
     <row r="265"/>
     <row r="266">
@@ -13888,6 +13394,11 @@
       <c r="S266" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T266" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -14007,21 +13518,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E268" t="inlineStr"/>
-      <c r="F268" t="inlineStr"/>
-      <c r="G268" t="inlineStr"/>
-      <c r="H268" t="inlineStr"/>
-      <c r="I268" t="inlineStr"/>
-      <c r="J268" t="inlineStr"/>
-      <c r="K268" t="inlineStr"/>
-      <c r="L268" t="inlineStr"/>
-      <c r="M268" t="inlineStr"/>
-      <c r="N268" t="inlineStr"/>
-      <c r="O268" t="inlineStr"/>
-      <c r="P268" t="inlineStr"/>
-      <c r="Q268" t="inlineStr"/>
-      <c r="R268" t="inlineStr"/>
-      <c r="S268" t="inlineStr"/>
     </row>
     <row r="269"/>
     <row r="270">
@@ -14090,6 +13586,11 @@
       <c r="S270" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T270" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -14209,21 +13710,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr"/>
-      <c r="F272" t="inlineStr"/>
-      <c r="G272" t="inlineStr"/>
-      <c r="H272" t="inlineStr"/>
-      <c r="I272" t="inlineStr"/>
-      <c r="J272" t="inlineStr"/>
-      <c r="K272" t="inlineStr"/>
-      <c r="L272" t="inlineStr"/>
-      <c r="M272" t="inlineStr"/>
-      <c r="N272" t="inlineStr"/>
-      <c r="O272" t="inlineStr"/>
-      <c r="P272" t="inlineStr"/>
-      <c r="Q272" t="inlineStr"/>
-      <c r="R272" t="inlineStr"/>
-      <c r="S272" t="inlineStr"/>
     </row>
     <row r="273"/>
     <row r="274">
@@ -14292,6 +13778,11 @@
       <c r="S274" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T274" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -14411,21 +13902,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E276" t="inlineStr"/>
-      <c r="F276" t="inlineStr"/>
-      <c r="G276" t="inlineStr"/>
-      <c r="H276" t="inlineStr"/>
-      <c r="I276" t="inlineStr"/>
-      <c r="J276" t="inlineStr"/>
-      <c r="K276" t="inlineStr"/>
-      <c r="L276" t="inlineStr"/>
-      <c r="M276" t="inlineStr"/>
-      <c r="N276" t="inlineStr"/>
-      <c r="O276" t="inlineStr"/>
-      <c r="P276" t="inlineStr"/>
-      <c r="Q276" t="inlineStr"/>
-      <c r="R276" t="inlineStr"/>
-      <c r="S276" t="inlineStr"/>
     </row>
     <row r="277"/>
     <row r="278">
@@ -14494,6 +13970,11 @@
       <c r="S278" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T278" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -14613,21 +14094,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E280" t="inlineStr"/>
-      <c r="F280" t="inlineStr"/>
-      <c r="G280" t="inlineStr"/>
-      <c r="H280" t="inlineStr"/>
-      <c r="I280" t="inlineStr"/>
-      <c r="J280" t="inlineStr"/>
-      <c r="K280" t="inlineStr"/>
-      <c r="L280" t="inlineStr"/>
-      <c r="M280" t="inlineStr"/>
-      <c r="N280" t="inlineStr"/>
-      <c r="O280" t="inlineStr"/>
-      <c r="P280" t="inlineStr"/>
-      <c r="Q280" t="inlineStr"/>
-      <c r="R280" t="inlineStr"/>
-      <c r="S280" t="inlineStr"/>
     </row>
     <row r="281"/>
     <row r="282">
@@ -14696,6 +14162,11 @@
       <c r="S282" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T282" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -14815,18 +14286,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E284" t="inlineStr"/>
-      <c r="F284" t="inlineStr"/>
-      <c r="G284" t="inlineStr"/>
-      <c r="H284" t="inlineStr"/>
-      <c r="I284" t="inlineStr"/>
-      <c r="J284" t="inlineStr"/>
-      <c r="K284" t="inlineStr"/>
-      <c r="L284" t="inlineStr"/>
-      <c r="M284" t="inlineStr"/>
-      <c r="N284" t="inlineStr"/>
-      <c r="O284" t="inlineStr"/>
-      <c r="P284" t="inlineStr"/>
       <c r="Q284" t="inlineStr">
         <is>
           <t>E</t>
@@ -14837,7 +14296,31 @@
           <t>I</t>
         </is>
       </c>
-      <c r="S284" t="inlineStr"/>
+      <c r="T284" t="inlineStr">
+        <is>
+          <r>
+            <t>D168E</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>65</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>V170I</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>65</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="285"/>
     <row r="286">
@@ -14906,6 +14389,11 @@
       <c r="S286" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T286" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -15025,25 +14513,24 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E288" t="inlineStr"/>
-      <c r="F288" t="inlineStr"/>
-      <c r="G288" t="inlineStr"/>
-      <c r="H288" t="inlineStr"/>
-      <c r="I288" t="inlineStr"/>
-      <c r="J288" t="inlineStr"/>
-      <c r="K288" t="inlineStr"/>
-      <c r="L288" t="inlineStr"/>
-      <c r="M288" t="inlineStr"/>
-      <c r="N288" t="inlineStr"/>
-      <c r="O288" t="inlineStr"/>
-      <c r="P288" t="inlineStr"/>
-      <c r="Q288" t="inlineStr"/>
       <c r="R288" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="S288" t="inlineStr"/>
+      <c r="T288" t="inlineStr">
+        <is>
+          <r>
+            <t>A170V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>83</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="289"/>
     <row r="290">
@@ -15112,6 +14599,11 @@
       <c r="S290" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T290" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -15231,21 +14723,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr"/>
-      <c r="F292" t="inlineStr"/>
-      <c r="G292" t="inlineStr"/>
-      <c r="H292" t="inlineStr"/>
-      <c r="I292" t="inlineStr"/>
-      <c r="J292" t="inlineStr"/>
-      <c r="K292" t="inlineStr"/>
-      <c r="L292" t="inlineStr"/>
-      <c r="M292" t="inlineStr"/>
-      <c r="N292" t="inlineStr"/>
-      <c r="O292" t="inlineStr"/>
-      <c r="P292" t="inlineStr"/>
-      <c r="Q292" t="inlineStr"/>
-      <c r="R292" t="inlineStr"/>
-      <c r="S292" t="inlineStr"/>
     </row>
     <row r="293"/>
     <row r="294">
@@ -15314,6 +14791,11 @@
       <c r="S294" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T294" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -15433,21 +14915,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E296" t="inlineStr"/>
-      <c r="F296" t="inlineStr"/>
-      <c r="G296" t="inlineStr"/>
-      <c r="H296" t="inlineStr"/>
-      <c r="I296" t="inlineStr"/>
-      <c r="J296" t="inlineStr"/>
-      <c r="K296" t="inlineStr"/>
-      <c r="L296" t="inlineStr"/>
-      <c r="M296" t="inlineStr"/>
-      <c r="N296" t="inlineStr"/>
-      <c r="O296" t="inlineStr"/>
-      <c r="P296" t="inlineStr"/>
-      <c r="Q296" t="inlineStr"/>
-      <c r="R296" t="inlineStr"/>
-      <c r="S296" t="inlineStr"/>
     </row>
     <row r="297"/>
     <row r="298">
@@ -15516,6 +14983,11 @@
       <c r="S298" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T298" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -15640,20 +15112,19 @@
           <t>L</t>
         </is>
       </c>
-      <c r="F300" t="inlineStr"/>
-      <c r="G300" t="inlineStr"/>
-      <c r="H300" t="inlineStr"/>
-      <c r="I300" t="inlineStr"/>
-      <c r="J300" t="inlineStr"/>
-      <c r="K300" t="inlineStr"/>
-      <c r="L300" t="inlineStr"/>
-      <c r="M300" t="inlineStr"/>
-      <c r="N300" t="inlineStr"/>
-      <c r="O300" t="inlineStr"/>
-      <c r="P300" t="inlineStr"/>
-      <c r="Q300" t="inlineStr"/>
-      <c r="R300" t="inlineStr"/>
-      <c r="S300" t="inlineStr"/>
+      <c r="T300" t="inlineStr">
+        <is>
+          <r>
+            <t>V36L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>50</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="301"/>
     <row r="302">
@@ -15722,6 +15193,11 @@
       <c r="S302" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T302" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -15841,25 +15317,24 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E304" t="inlineStr"/>
-      <c r="F304" t="inlineStr"/>
-      <c r="G304" t="inlineStr"/>
-      <c r="H304" t="inlineStr"/>
-      <c r="I304" t="inlineStr"/>
-      <c r="J304" t="inlineStr"/>
-      <c r="K304" t="inlineStr"/>
       <c r="L304" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="M304" t="inlineStr"/>
-      <c r="N304" t="inlineStr"/>
-      <c r="O304" t="inlineStr"/>
-      <c r="P304" t="inlineStr"/>
-      <c r="Q304" t="inlineStr"/>
-      <c r="R304" t="inlineStr"/>
-      <c r="S304" t="inlineStr"/>
+      <c r="T304" t="inlineStr">
+        <is>
+          <r>
+            <t>S122T</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>75</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="305"/>
     <row r="306">
@@ -15928,6 +15403,11 @@
       <c r="S306" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T306" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -16047,21 +15527,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E308" t="inlineStr"/>
-      <c r="F308" t="inlineStr"/>
-      <c r="G308" t="inlineStr"/>
-      <c r="H308" t="inlineStr"/>
-      <c r="I308" t="inlineStr"/>
-      <c r="J308" t="inlineStr"/>
-      <c r="K308" t="inlineStr"/>
-      <c r="L308" t="inlineStr"/>
-      <c r="M308" t="inlineStr"/>
-      <c r="N308" t="inlineStr"/>
-      <c r="O308" t="inlineStr"/>
-      <c r="P308" t="inlineStr"/>
-      <c r="Q308" t="inlineStr"/>
-      <c r="R308" t="inlineStr"/>
-      <c r="S308" t="inlineStr"/>
     </row>
     <row r="309"/>
     <row r="310">
@@ -16130,6 +15595,11 @@
       <c r="S310" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T310" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -16249,21 +15719,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E312" t="inlineStr"/>
-      <c r="F312" t="inlineStr"/>
-      <c r="G312" t="inlineStr"/>
-      <c r="H312" t="inlineStr"/>
-      <c r="I312" t="inlineStr"/>
-      <c r="J312" t="inlineStr"/>
-      <c r="K312" t="inlineStr"/>
-      <c r="L312" t="inlineStr"/>
-      <c r="M312" t="inlineStr"/>
-      <c r="N312" t="inlineStr"/>
-      <c r="O312" t="inlineStr"/>
-      <c r="P312" t="inlineStr"/>
-      <c r="Q312" t="inlineStr"/>
-      <c r="R312" t="inlineStr"/>
-      <c r="S312" t="inlineStr"/>
     </row>
     <row r="313"/>
     <row r="314">
@@ -16332,6 +15787,11 @@
       <c r="S314" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T314" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -16451,21 +15911,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E316" t="inlineStr"/>
-      <c r="F316" t="inlineStr"/>
-      <c r="G316" t="inlineStr"/>
-      <c r="H316" t="inlineStr"/>
-      <c r="I316" t="inlineStr"/>
-      <c r="J316" t="inlineStr"/>
-      <c r="K316" t="inlineStr"/>
-      <c r="L316" t="inlineStr"/>
-      <c r="M316" t="inlineStr"/>
-      <c r="N316" t="inlineStr"/>
-      <c r="O316" t="inlineStr"/>
-      <c r="P316" t="inlineStr"/>
-      <c r="Q316" t="inlineStr"/>
-      <c r="R316" t="inlineStr"/>
-      <c r="S316" t="inlineStr"/>
     </row>
     <row r="317"/>
     <row r="318">
@@ -16534,6 +15979,11 @@
       <c r="S318" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T318" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -16653,21 +16103,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E320" t="inlineStr"/>
-      <c r="F320" t="inlineStr"/>
-      <c r="G320" t="inlineStr"/>
-      <c r="H320" t="inlineStr"/>
-      <c r="I320" t="inlineStr"/>
-      <c r="J320" t="inlineStr"/>
-      <c r="K320" t="inlineStr"/>
-      <c r="L320" t="inlineStr"/>
-      <c r="M320" t="inlineStr"/>
-      <c r="N320" t="inlineStr"/>
-      <c r="O320" t="inlineStr"/>
-      <c r="P320" t="inlineStr"/>
-      <c r="Q320" t="inlineStr"/>
-      <c r="R320" t="inlineStr"/>
-      <c r="S320" t="inlineStr"/>
     </row>
     <row r="321"/>
     <row r="322">
@@ -16736,6 +16171,11 @@
       <c r="S322" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T322" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -16855,21 +16295,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E324" t="inlineStr"/>
-      <c r="F324" t="inlineStr"/>
-      <c r="G324" t="inlineStr"/>
-      <c r="H324" t="inlineStr"/>
-      <c r="I324" t="inlineStr"/>
-      <c r="J324" t="inlineStr"/>
-      <c r="K324" t="inlineStr"/>
-      <c r="L324" t="inlineStr"/>
-      <c r="M324" t="inlineStr"/>
-      <c r="N324" t="inlineStr"/>
-      <c r="O324" t="inlineStr"/>
-      <c r="P324" t="inlineStr"/>
-      <c r="Q324" t="inlineStr"/>
-      <c r="R324" t="inlineStr"/>
-      <c r="S324" t="inlineStr"/>
     </row>
     <row r="325"/>
     <row r="326">
@@ -16938,6 +16363,11 @@
       <c r="S326" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T326" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -17057,21 +16487,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E328" t="inlineStr"/>
-      <c r="F328" t="inlineStr"/>
-      <c r="G328" t="inlineStr"/>
-      <c r="H328" t="inlineStr"/>
-      <c r="I328" t="inlineStr"/>
-      <c r="J328" t="inlineStr"/>
-      <c r="K328" t="inlineStr"/>
-      <c r="L328" t="inlineStr"/>
-      <c r="M328" t="inlineStr"/>
-      <c r="N328" t="inlineStr"/>
-      <c r="O328" t="inlineStr"/>
-      <c r="P328" t="inlineStr"/>
-      <c r="Q328" t="inlineStr"/>
-      <c r="R328" t="inlineStr"/>
-      <c r="S328" t="inlineStr"/>
     </row>
     <row r="329"/>
     <row r="330">
@@ -17140,6 +16555,11 @@
       <c r="S330" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T330" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -17259,21 +16679,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr"/>
-      <c r="F332" t="inlineStr"/>
-      <c r="G332" t="inlineStr"/>
-      <c r="H332" t="inlineStr"/>
-      <c r="I332" t="inlineStr"/>
-      <c r="J332" t="inlineStr"/>
-      <c r="K332" t="inlineStr"/>
-      <c r="L332" t="inlineStr"/>
-      <c r="M332" t="inlineStr"/>
-      <c r="N332" t="inlineStr"/>
-      <c r="O332" t="inlineStr"/>
-      <c r="P332" t="inlineStr"/>
-      <c r="Q332" t="inlineStr"/>
-      <c r="R332" t="inlineStr"/>
-      <c r="S332" t="inlineStr"/>
     </row>
     <row r="333"/>
     <row r="334">
@@ -17342,6 +16747,11 @@
       <c r="S334" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T334" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -17461,21 +16871,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E336" t="inlineStr"/>
-      <c r="F336" t="inlineStr"/>
-      <c r="G336" t="inlineStr"/>
-      <c r="H336" t="inlineStr"/>
-      <c r="I336" t="inlineStr"/>
-      <c r="J336" t="inlineStr"/>
-      <c r="K336" t="inlineStr"/>
-      <c r="L336" t="inlineStr"/>
-      <c r="M336" t="inlineStr"/>
-      <c r="N336" t="inlineStr"/>
-      <c r="O336" t="inlineStr"/>
-      <c r="P336" t="inlineStr"/>
-      <c r="Q336" t="inlineStr"/>
-      <c r="R336" t="inlineStr"/>
-      <c r="S336" t="inlineStr"/>
     </row>
     <row r="337"/>
     <row r="338">
@@ -17544,6 +16939,11 @@
       <c r="S338" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T338" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -17663,21 +17063,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E340" t="inlineStr"/>
-      <c r="F340" t="inlineStr"/>
-      <c r="G340" t="inlineStr"/>
-      <c r="H340" t="inlineStr"/>
-      <c r="I340" t="inlineStr"/>
-      <c r="J340" t="inlineStr"/>
-      <c r="K340" t="inlineStr"/>
-      <c r="L340" t="inlineStr"/>
-      <c r="M340" t="inlineStr"/>
-      <c r="N340" t="inlineStr"/>
-      <c r="O340" t="inlineStr"/>
-      <c r="P340" t="inlineStr"/>
-      <c r="Q340" t="inlineStr"/>
-      <c r="R340" t="inlineStr"/>
-      <c r="S340" t="inlineStr"/>
     </row>
     <row r="341"/>
     <row r="342">
@@ -17746,6 +17131,11 @@
       <c r="S342" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T342" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -17865,25 +17255,24 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E344" t="inlineStr"/>
-      <c r="F344" t="inlineStr"/>
-      <c r="G344" t="inlineStr"/>
-      <c r="H344" t="inlineStr"/>
-      <c r="I344" t="inlineStr"/>
       <c r="J344" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="K344" t="inlineStr"/>
-      <c r="L344" t="inlineStr"/>
-      <c r="M344" t="inlineStr"/>
-      <c r="N344" t="inlineStr"/>
-      <c r="O344" t="inlineStr"/>
-      <c r="P344" t="inlineStr"/>
-      <c r="Q344" t="inlineStr"/>
-      <c r="R344" t="inlineStr"/>
-      <c r="S344" t="inlineStr"/>
+      <c r="T344" t="inlineStr">
+        <is>
+          <r>
+            <t>F56Y</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>60</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="345"/>
     <row r="346">
@@ -17952,6 +17341,11 @@
       <c r="S346" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T346" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -18071,21 +17465,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E348" t="inlineStr"/>
-      <c r="F348" t="inlineStr"/>
-      <c r="G348" t="inlineStr"/>
-      <c r="H348" t="inlineStr"/>
-      <c r="I348" t="inlineStr"/>
-      <c r="J348" t="inlineStr"/>
-      <c r="K348" t="inlineStr"/>
-      <c r="L348" t="inlineStr"/>
-      <c r="M348" t="inlineStr"/>
-      <c r="N348" t="inlineStr"/>
-      <c r="O348" t="inlineStr"/>
-      <c r="P348" t="inlineStr"/>
-      <c r="Q348" t="inlineStr"/>
-      <c r="R348" t="inlineStr"/>
-      <c r="S348" t="inlineStr"/>
     </row>
     <row r="349"/>
     <row r="350">
@@ -18154,6 +17533,11 @@
       <c r="S350" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T350" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -18273,21 +17657,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E352" t="inlineStr"/>
-      <c r="F352" t="inlineStr"/>
-      <c r="G352" t="inlineStr"/>
-      <c r="H352" t="inlineStr"/>
-      <c r="I352" t="inlineStr"/>
-      <c r="J352" t="inlineStr"/>
-      <c r="K352" t="inlineStr"/>
-      <c r="L352" t="inlineStr"/>
-      <c r="M352" t="inlineStr"/>
-      <c r="N352" t="inlineStr"/>
-      <c r="O352" t="inlineStr"/>
-      <c r="P352" t="inlineStr"/>
-      <c r="Q352" t="inlineStr"/>
-      <c r="R352" t="inlineStr"/>
-      <c r="S352" t="inlineStr"/>
     </row>
     <row r="353"/>
     <row r="354">
@@ -18356,6 +17725,11 @@
       <c r="S354" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T354" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -18475,21 +17849,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E356" t="inlineStr"/>
-      <c r="F356" t="inlineStr"/>
-      <c r="G356" t="inlineStr"/>
-      <c r="H356" t="inlineStr"/>
-      <c r="I356" t="inlineStr"/>
-      <c r="J356" t="inlineStr"/>
-      <c r="K356" t="inlineStr"/>
-      <c r="L356" t="inlineStr"/>
-      <c r="M356" t="inlineStr"/>
-      <c r="N356" t="inlineStr"/>
-      <c r="O356" t="inlineStr"/>
-      <c r="P356" t="inlineStr"/>
-      <c r="Q356" t="inlineStr"/>
-      <c r="R356" t="inlineStr"/>
-      <c r="S356" t="inlineStr"/>
     </row>
     <row r="357"/>
     <row r="358">
@@ -18558,6 +17917,11 @@
       <c r="S358" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T358" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -18682,24 +18046,36 @@
           <t>V</t>
         </is>
       </c>
-      <c r="F360" t="inlineStr"/>
-      <c r="G360" t="inlineStr"/>
-      <c r="H360" t="inlineStr"/>
-      <c r="I360" t="inlineStr"/>
-      <c r="J360" t="inlineStr"/>
-      <c r="K360" t="inlineStr"/>
-      <c r="L360" t="inlineStr"/>
-      <c r="M360" t="inlineStr"/>
-      <c r="N360" t="inlineStr"/>
       <c r="O360" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="P360" t="inlineStr"/>
-      <c r="Q360" t="inlineStr"/>
-      <c r="R360" t="inlineStr"/>
-      <c r="S360" t="inlineStr"/>
+      <c r="T360" t="inlineStr">
+        <is>
+          <r>
+            <t>L36V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>32</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>I158V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>95</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="361"/>
     <row r="362">
@@ -18768,6 +18144,11 @@
       <c r="S362" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T362" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -18892,20 +18273,19 @@
           <t>V</t>
         </is>
       </c>
-      <c r="F364" t="inlineStr"/>
-      <c r="G364" t="inlineStr"/>
-      <c r="H364" t="inlineStr"/>
-      <c r="I364" t="inlineStr"/>
-      <c r="J364" t="inlineStr"/>
-      <c r="K364" t="inlineStr"/>
-      <c r="L364" t="inlineStr"/>
-      <c r="M364" t="inlineStr"/>
-      <c r="N364" t="inlineStr"/>
-      <c r="O364" t="inlineStr"/>
-      <c r="P364" t="inlineStr"/>
-      <c r="Q364" t="inlineStr"/>
-      <c r="R364" t="inlineStr"/>
-      <c r="S364" t="inlineStr"/>
+      <c r="T364" t="inlineStr">
+        <is>
+          <r>
+            <t>L36V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>32</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="365"/>
     <row r="366">
@@ -18974,6 +18354,11 @@
       <c r="S366" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T366" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -19093,21 +18478,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E368" t="inlineStr"/>
-      <c r="F368" t="inlineStr"/>
-      <c r="G368" t="inlineStr"/>
-      <c r="H368" t="inlineStr"/>
-      <c r="I368" t="inlineStr"/>
-      <c r="J368" t="inlineStr"/>
-      <c r="K368" t="inlineStr"/>
-      <c r="L368" t="inlineStr"/>
-      <c r="M368" t="inlineStr"/>
-      <c r="N368" t="inlineStr"/>
-      <c r="O368" t="inlineStr"/>
-      <c r="P368" t="inlineStr"/>
-      <c r="Q368" t="inlineStr"/>
-      <c r="R368" t="inlineStr"/>
-      <c r="S368" t="inlineStr"/>
     </row>
     <row r="369"/>
     <row r="370">
@@ -19176,6 +18546,11 @@
       <c r="S370" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T370" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -19295,21 +18670,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E372" t="inlineStr"/>
-      <c r="F372" t="inlineStr"/>
-      <c r="G372" t="inlineStr"/>
-      <c r="H372" t="inlineStr"/>
-      <c r="I372" t="inlineStr"/>
-      <c r="J372" t="inlineStr"/>
-      <c r="K372" t="inlineStr"/>
-      <c r="L372" t="inlineStr"/>
-      <c r="M372" t="inlineStr"/>
-      <c r="N372" t="inlineStr"/>
-      <c r="O372" t="inlineStr"/>
-      <c r="P372" t="inlineStr"/>
-      <c r="Q372" t="inlineStr"/>
-      <c r="R372" t="inlineStr"/>
-      <c r="S372" t="inlineStr"/>
     </row>
     <row r="373"/>
     <row r="374">
@@ -19378,6 +18738,11 @@
       <c r="S374" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T374" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -19497,21 +18862,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E376" t="inlineStr"/>
-      <c r="F376" t="inlineStr"/>
-      <c r="G376" t="inlineStr"/>
-      <c r="H376" t="inlineStr"/>
-      <c r="I376" t="inlineStr"/>
-      <c r="J376" t="inlineStr"/>
-      <c r="K376" t="inlineStr"/>
-      <c r="L376" t="inlineStr"/>
-      <c r="M376" t="inlineStr"/>
-      <c r="N376" t="inlineStr"/>
-      <c r="O376" t="inlineStr"/>
-      <c r="P376" t="inlineStr"/>
-      <c r="Q376" t="inlineStr"/>
-      <c r="R376" t="inlineStr"/>
-      <c r="S376" t="inlineStr"/>
     </row>
     <row r="377"/>
     <row r="378">
@@ -19580,6 +18930,11 @@
       <c r="S378" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T378" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -19667,7 +19022,6 @@
           <t>Q</t>
         </is>
       </c>
-      <c r="R379" t="inlineStr"/>
       <c r="S379" t="inlineStr">
         <is>
           <t>L</t>
@@ -19695,9 +19049,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E380" t="inlineStr"/>
-      <c r="F380" t="inlineStr"/>
-      <c r="G380" t="inlineStr"/>
       <c r="H380" t="inlineStr">
         <is>
           <t>A</t>
@@ -19708,22 +19059,63 @@
           <t>P</t>
         </is>
       </c>
-      <c r="J380" t="inlineStr"/>
-      <c r="K380" t="inlineStr"/>
       <c r="L380" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M380" t="inlineStr"/>
-      <c r="N380" t="inlineStr"/>
-      <c r="O380" t="inlineStr"/>
-      <c r="P380" t="inlineStr"/>
-      <c r="Q380" t="inlineStr"/>
-      <c r="R380" t="inlineStr"/>
       <c r="S380" t="inlineStr">
         <is>
           <t>M</t>
+        </is>
+      </c>
+      <c r="T380" t="inlineStr">
+        <is>
+          <r>
+            <t>S54A</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>V55P</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>K122N</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L175M</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
         </is>
       </c>
     </row>
@@ -19794,6 +19186,11 @@
       <c r="S382" s="1" t="n">
         <v>175</v>
       </c>
+      <c r="T382" s="1" t="inlineStr">
+        <is>
+          <t>Mutations</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -19913,21 +19310,6 @@
           <t>Consensus</t>
         </is>
       </c>
-      <c r="E384" t="inlineStr"/>
-      <c r="F384" t="inlineStr"/>
-      <c r="G384" t="inlineStr"/>
-      <c r="H384" t="inlineStr"/>
-      <c r="I384" t="inlineStr"/>
-      <c r="J384" t="inlineStr"/>
-      <c r="K384" t="inlineStr"/>
-      <c r="L384" t="inlineStr"/>
-      <c r="M384" t="inlineStr"/>
-      <c r="N384" t="inlineStr"/>
-      <c r="O384" t="inlineStr"/>
-      <c r="P384" t="inlineStr"/>
-      <c r="Q384" t="inlineStr"/>
-      <c r="R384" t="inlineStr"/>
-      <c r="S384" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refresh COMET subtype consensus comparisons
</commit_message>
<xml_diff>
--- a/Reference_seqs/HCV_Subtype_Ref_vs_Comet_Subtype_Consensus_Aligned_NS3.xlsx
+++ b/Reference_seqs/HCV_Subtype_Ref_vs_Comet_Subtype_Consensus_Aligned_NS3.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T384"/>
+  <dimension ref="A1:T380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18862,450 +18862,212 @@
           <t>Consensus</t>
         </is>
       </c>
-    </row>
-    <row r="377"/>
-    <row r="378">
-      <c r="A378" s="1" t="inlineStr">
-        <is>
-          <t>Gene</t>
-        </is>
-      </c>
-      <c r="B378" s="1" t="inlineStr">
-        <is>
-          <t>Genotype</t>
-        </is>
-      </c>
-      <c r="C378" s="1" t="inlineStr">
-        <is>
-          <t>Subtype</t>
-        </is>
-      </c>
-      <c r="D378" s="1" t="inlineStr">
-        <is>
-          <t>Sequence</t>
-        </is>
-      </c>
-      <c r="E378" s="1" t="n">
-        <v>36</v>
-      </c>
-      <c r="F378" s="1" t="n">
-        <v>41</v>
-      </c>
-      <c r="G378" s="1" t="n">
-        <v>43</v>
-      </c>
-      <c r="H378" s="1" t="n">
-        <v>54</v>
-      </c>
-      <c r="I378" s="1" t="n">
-        <v>55</v>
-      </c>
-      <c r="J378" s="1" t="n">
-        <v>56</v>
-      </c>
-      <c r="K378" s="1" t="n">
-        <v>80</v>
-      </c>
-      <c r="L378" s="1" t="n">
-        <v>122</v>
-      </c>
-      <c r="M378" s="1" t="n">
-        <v>155</v>
-      </c>
-      <c r="N378" s="1" t="n">
-        <v>156</v>
-      </c>
-      <c r="O378" s="1" t="n">
-        <v>158</v>
-      </c>
-      <c r="P378" s="1" t="n">
-        <v>166</v>
-      </c>
-      <c r="Q378" s="1" t="n">
-        <v>168</v>
-      </c>
-      <c r="R378" s="1" t="n">
-        <v>170</v>
-      </c>
-      <c r="S378" s="1" t="n">
-        <v>175</v>
-      </c>
-      <c r="T378" s="1" t="inlineStr">
-        <is>
-          <t>Mutations</t>
-        </is>
-      </c>
-    </row>
-    <row r="379">
-      <c r="A379" t="inlineStr">
-        <is>
-          <t>NS3</t>
-        </is>
-      </c>
-      <c r="B379" t="inlineStr">
-        <is>
-          <t>GT7</t>
-        </is>
-      </c>
-      <c r="C379" t="inlineStr">
-        <is>
-          <t>7b</t>
-        </is>
-      </c>
-      <c r="D379" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="E379" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="F379" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="G379" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="H379" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I379" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="J379" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="K379" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="L379" t="inlineStr">
-        <is>
-          <t>K</t>
-        </is>
-      </c>
-      <c r="M379" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="N379" t="inlineStr">
+      <c r="H376" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="O379" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="P379" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="Q379" t="inlineStr">
-        <is>
-          <t>Q</t>
-        </is>
-      </c>
-      <c r="S379" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-    </row>
-    <row r="380">
-      <c r="A380" t="inlineStr">
-        <is>
-          <t>NS3</t>
-        </is>
-      </c>
-      <c r="B380" t="inlineStr">
-        <is>
-          <t>GT7</t>
-        </is>
-      </c>
-      <c r="C380" t="inlineStr">
-        <is>
-          <t>7b</t>
-        </is>
-      </c>
-      <c r="D380" t="inlineStr">
-        <is>
-          <t>Consensus</t>
-        </is>
-      </c>
-      <c r="H380" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="I380" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L380" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="S380" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="T380" t="inlineStr">
+      <c r="T376" t="inlineStr">
         <is>
           <r>
-            <t>S54A</t>
+            <t>G54A</t>
           </r>
           <r>
             <rPr>
               <vertAlign val="subscript"/>
             </rPr>
-            <t>100</t>
+            <t>50</t>
           </r>
-          <r>
-            <t xml:space="preserve">, </t>
-          </r>
-          <r>
-            <t>V55P</t>
-          </r>
-          <r>
-            <rPr>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>100</t>
-          </r>
-          <r>
-            <t xml:space="preserve">, </t>
-          </r>
-          <r>
-            <t>K122N</t>
-          </r>
-          <r>
-            <rPr>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>100</t>
-          </r>
-          <r>
-            <t xml:space="preserve">, </t>
-          </r>
-          <r>
-            <t>L175M</t>
-          </r>
-          <r>
-            <rPr>
-              <vertAlign val="subscript"/>
-            </rPr>
-            <t>100</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="381"/>
-    <row r="382">
-      <c r="A382" s="1" t="inlineStr">
+        </is>
+      </c>
+    </row>
+    <row r="377"/>
+    <row r="378">
+      <c r="A378" s="1" t="inlineStr">
         <is>
           <t>Gene</t>
         </is>
       </c>
-      <c r="B382" s="1" t="inlineStr">
+      <c r="B378" s="1" t="inlineStr">
         <is>
           <t>Genotype</t>
         </is>
       </c>
-      <c r="C382" s="1" t="inlineStr">
+      <c r="C378" s="1" t="inlineStr">
         <is>
           <t>Subtype</t>
         </is>
       </c>
-      <c r="D382" s="1" t="inlineStr">
+      <c r="D378" s="1" t="inlineStr">
         <is>
           <t>Sequence</t>
         </is>
       </c>
-      <c r="E382" s="1" t="n">
+      <c r="E378" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="F382" s="1" t="n">
+      <c r="F378" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="G382" s="1" t="n">
+      <c r="G378" s="1" t="n">
         <v>43</v>
       </c>
-      <c r="H382" s="1" t="n">
+      <c r="H378" s="1" t="n">
         <v>54</v>
       </c>
-      <c r="I382" s="1" t="n">
+      <c r="I378" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="J382" s="1" t="n">
+      <c r="J378" s="1" t="n">
         <v>56</v>
       </c>
-      <c r="K382" s="1" t="n">
+      <c r="K378" s="1" t="n">
         <v>80</v>
       </c>
-      <c r="L382" s="1" t="n">
+      <c r="L378" s="1" t="n">
         <v>122</v>
       </c>
-      <c r="M382" s="1" t="n">
+      <c r="M378" s="1" t="n">
         <v>155</v>
       </c>
-      <c r="N382" s="1" t="n">
+      <c r="N378" s="1" t="n">
         <v>156</v>
       </c>
-      <c r="O382" s="1" t="n">
+      <c r="O378" s="1" t="n">
         <v>158</v>
       </c>
-      <c r="P382" s="1" t="n">
+      <c r="P378" s="1" t="n">
         <v>166</v>
       </c>
-      <c r="Q382" s="1" t="n">
+      <c r="Q378" s="1" t="n">
         <v>168</v>
       </c>
-      <c r="R382" s="1" t="n">
+      <c r="R378" s="1" t="n">
         <v>170</v>
       </c>
-      <c r="S382" s="1" t="n">
+      <c r="S378" s="1" t="n">
         <v>175</v>
       </c>
-      <c r="T382" s="1" t="inlineStr">
+      <c r="T378" s="1" t="inlineStr">
         <is>
           <t>Mutations</t>
         </is>
       </c>
     </row>
-    <row r="383">
-      <c r="A383" t="inlineStr">
+    <row r="379">
+      <c r="A379" t="inlineStr">
         <is>
           <t>NS3</t>
         </is>
       </c>
-      <c r="B383" t="inlineStr">
+      <c r="B379" t="inlineStr">
         <is>
           <t>GT8</t>
         </is>
       </c>
-      <c r="C383" t="inlineStr">
+      <c r="C379" t="inlineStr">
         <is>
           <t>8a</t>
         </is>
       </c>
-      <c r="D383" t="inlineStr">
+      <c r="D379" t="inlineStr">
         <is>
           <t>Reference</t>
         </is>
       </c>
-      <c r="E383" t="inlineStr">
+      <c r="E379" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="F383" t="inlineStr">
+      <c r="F379" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G383" t="inlineStr">
+      <c r="G379" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="H383" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="I383" t="inlineStr">
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="J383" t="inlineStr">
+      <c r="J379" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="K383" t="inlineStr">
+      <c r="K379" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="L383" t="inlineStr">
+      <c r="L379" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="M383" t="inlineStr">
+      <c r="M379" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="N383" t="inlineStr">
+      <c r="N379" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="O383" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="P383" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="Q383" t="inlineStr">
+      <c r="O379" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P379" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="Q379" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="R383" t="inlineStr">
+      <c r="R379" t="inlineStr">
         <is>
           <t>P</t>
         </is>
       </c>
-      <c r="S383" t="inlineStr">
+      <c r="S379" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
     </row>
-    <row r="384">
-      <c r="A384" t="inlineStr">
+    <row r="380">
+      <c r="A380" t="inlineStr">
         <is>
           <t>NS3</t>
         </is>
       </c>
-      <c r="B384" t="inlineStr">
+      <c r="B380" t="inlineStr">
         <is>
           <t>GT8</t>
         </is>
       </c>
-      <c r="C384" t="inlineStr">
+      <c r="C380" t="inlineStr">
         <is>
           <t>8a</t>
         </is>
       </c>
-      <c r="D384" t="inlineStr">
+      <c r="D380" t="inlineStr">
         <is>
           <t>Consensus</t>
         </is>

</xml_diff>

<commit_message>
Preserve consensus coordinates and add coverage audit
</commit_message>
<xml_diff>
--- a/Reference_seqs/HCV_Subtype_Ref_vs_Comet_Subtype_Consensus_Aligned_NS3.xlsx
+++ b/Reference_seqs/HCV_Subtype_Ref_vs_Comet_Subtype_Consensus_Aligned_NS3.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RAS comparison" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAS comparison" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6883,6 +6883,245 @@
           <t>Consensus</t>
         </is>
       </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q132" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <r>
+            <t>S36L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T41Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L43F</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>V54T</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>99</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>Y55V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>H56Y</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>D80Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>99</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T122S</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>99</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>A155R</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>94</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>C158V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>99</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L166A</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>98</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>F168Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>P170I</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>S175L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="133"/>
     <row r="134">
@@ -7075,6 +7314,245 @@
           <t>Consensus</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <r>
+            <t>S36L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T41Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L43F</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>V54T</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>Y55V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>H56Y</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>D80Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T122S</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>A155R</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>C158V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L166S</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>80</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>F168Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>P170I</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>S175L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="137"/>
     <row r="138">
@@ -7267,21 +7745,242 @@
           <t>Consensus</t>
         </is>
       </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
         <is>
           <r>
-            <t>N175S</t>
+            <t>S36L</t>
           </r>
           <r>
             <rPr>
               <vertAlign val="subscript"/>
             </rPr>
-            <t>NA</t>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T41Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L43F</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>V54T</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>Y55V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>H56Y</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>D80Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T122S</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>A155R</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>C158V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L166S</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>80</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>F168Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>P170I</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>N175L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
           </r>
         </is>
       </c>
@@ -7687,6 +8386,245 @@
           <t>Consensus</t>
         </is>
       </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <r>
+            <t>S36L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T41Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L43F</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>V54T</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>Y55V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>H56Y</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>D80Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>80</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T122S</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>A155R</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>C158V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L166A</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>F168Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>P170V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>A175L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="149"/>
     <row r="150">
@@ -7877,6 +8815,245 @@
       <c r="D152" t="inlineStr">
         <is>
           <t>Consensus</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <r>
+            <t>S36L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T41Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L43F</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>V54T</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>Y55V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>H56Y</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>D80Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>80</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>T122S</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>A155R</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>C158V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L166A</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>F168Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>P170V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>A175L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
         </is>
       </c>
     </row>
@@ -19072,6 +20249,228 @@
           <t>Consensus</t>
         </is>
       </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="P380" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Q380" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="R380" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="S380" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="T380" t="inlineStr">
+        <is>
+          <r>
+            <t>S36L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>S41Q</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>L43F</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>V54T</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>Y55V</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>H56Y</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>D80K</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>50</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>R122T</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>88</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>A155R</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>V166A</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>100</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>F168D</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>75</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>P170I</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>71</t>
+          </r>
+          <r>
+            <t xml:space="preserve">, </t>
+          </r>
+          <r>
+            <t>E175L</t>
+          </r>
+          <r>
+            <rPr>
+              <vertAlign val="subscript"/>
+            </rPr>
+            <t>71</t>
+          </r>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>